<commit_message>
corrected settings.py file and filize that
</commit_message>
<xml_diff>
--- a/TP_and_Preprocessing/onebridgeVerification/bridge_01577A016_04612_2025_elements.xlsx
+++ b/TP_and_Preprocessing/onebridgeVerification/bridge_01577A016_04612_2025_elements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\PSU\Projects\PhD\WeeklyMeetings_Tasks\24_04062026_BHI_RL\risk-based-bhi-softtree-ppo\TP_and_Preprocessing\onebridgeVerification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8AA4347-EDC5-4661-B41E-29E0080A97B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CADC19-DECD-43DB-A570-AF6A23873A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="37920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
first version for bridge_bhi_trainingtBHI.py
</commit_message>
<xml_diff>
--- a/TP_and_Preprocessing/onebridgeVerification/bridge_01577A016_04612_2025_elements.xlsx
+++ b/TP_and_Preprocessing/onebridgeVerification/bridge_01577A016_04612_2025_elements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\PSU\Projects\PhD\WeeklyMeetings_Tasks\24_04062026_BHI_RL\risk-based-bhi-softtree-ppo\TP_and_Preprocessing\onebridgeVerification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CADC19-DECD-43DB-A570-AF6A23873A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C235B3A-29D0-48EE-96C7-513AAB936047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="37920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -581,6 +581,7 @@
         <v>3</v>
       </c>
       <c r="G2">
+        <f>E2*F2</f>
         <v>6</v>
       </c>
       <c r="H2">
@@ -639,6 +640,7 @@
         <v>4</v>
       </c>
       <c r="G3">
+        <f t="shared" ref="G3:G10" si="0">E3*F3</f>
         <v>4</v>
       </c>
       <c r="H3">
@@ -669,7 +671,7 @@
         <v>0</v>
       </c>
       <c r="Q3">
-        <f t="shared" ref="Q3:Q10" si="0">(M3*I3+N3*J3+O3*K3+P3*L3)/H3</f>
+        <f t="shared" ref="Q3:Q10" si="1">(M3*I3+N3*J3+O3*K3+P3*L3)/H3</f>
         <v>0.99944908180300496</v>
       </c>
     </row>
@@ -693,6 +695,7 @@
         <v>4</v>
       </c>
       <c r="G4">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="H4">
@@ -723,7 +726,7 @@
         <v>0</v>
       </c>
       <c r="Q4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.83499999999999996</v>
       </c>
     </row>
@@ -747,6 +750,7 @@
         <v>2</v>
       </c>
       <c r="G5">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="H5">
@@ -777,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="Q5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.98730769230769233</v>
       </c>
     </row>
@@ -801,6 +805,7 @@
         <v>4</v>
       </c>
       <c r="G6">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="H6">
@@ -831,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.97461538461538455</v>
       </c>
     </row>
@@ -855,6 +860,7 @@
         <v>1</v>
       </c>
       <c r="G7">
+        <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
       <c r="H7">
@@ -885,7 +891,7 @@
         <v>0</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.84802631578947374</v>
       </c>
     </row>
@@ -909,6 +915,7 @@
         <v>3</v>
       </c>
       <c r="G8">
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
       <c r="H8">
@@ -939,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="Q8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -963,6 +970,7 @@
         <v>1</v>
       </c>
       <c r="G9">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="H9">
@@ -993,7 +1001,7 @@
         <v>0</v>
       </c>
       <c r="Q9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.90604436229205176</v>
       </c>
     </row>
@@ -1017,6 +1025,7 @@
         <v>1</v>
       </c>
       <c r="G10">
+        <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
       <c r="H10">
@@ -1047,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="Q10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.88792011344835731</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add verify_bhi_50_years.py and modify the  bridge_bhi_validation_obtBHI.py file to show the leaf and internal node corectly
</commit_message>
<xml_diff>
--- a/TP_and_Preprocessing/onebridgeVerification/bridge_01577A016_04612_2025_elements.xlsx
+++ b/TP_and_Preprocessing/onebridgeVerification/bridge_01577A016_04612_2025_elements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\PSU\Projects\PhD\WeeklyMeetings_Tasks\24_04062026_BHI_RL\risk-based-bhi-softtree-ppo\TP_and_Preprocessing\onebridgeVerification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C235B3A-29D0-48EE-96C7-513AAB936047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DFC034-966C-4D8C-8103-59D40FB4141E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="37920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17172" yWindow="7692" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>